<commit_message>
updated model and predictions
</commit_message>
<xml_diff>
--- a/data/Exam Study Habits Survey (Responses).xlsx
+++ b/data/Exam Study Habits Survey (Responses).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="94">
   <si>
     <t>Timestamp</t>
   </si>
@@ -284,6 +284,15 @@
   </si>
   <si>
     <t>Grainger Library, CIF, Funk Library, Siebel Center for CS, BIF, I school</t>
+  </si>
+  <si>
+    <t>Information Management</t>
+  </si>
+  <si>
+    <t>Grainger Library, CIF, Funk Library, Your Dorm/Apartment</t>
+  </si>
+  <si>
+    <t>Grainger Library, Illini Union, BIF, ECE Building, Your Dorm/Apartment</t>
   </si>
 </sst>
 </file>
@@ -421,7 +430,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:N30" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:N32" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="14">
     <tableColumn name="Timestamp" id="1"/>
     <tableColumn name="Major" id="2"/>
@@ -1786,6 +1795,82 @@
         <v>64</v>
       </c>
     </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="5">
+        <v>46133.60970947916</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D31" s="6">
+        <v>2027.0</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="L31" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="5">
+        <v>46134.43062853009</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="6">
+        <v>2028.0</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="K32" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L32" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M32" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>